<commit_message>
add IRIs to data
</commit_message>
<xml_diff>
--- a/data/raw/BookEdition.xlsx
+++ b/data/raw/BookEdition.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemivillars-amberg/Documents/daschland-scripts/data/spreadsheets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noraammann/Documents/Cloned_GitHub/daschland-scripts/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEFB682C-D062-434D-BA0D-9B6B52C6527D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59F74799-3F80-3D4E-B358-60F4275FEFFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="62900" windowHeight="21580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="44">
   <si>
     <t>ID</t>
   </si>
@@ -174,6 +173,12 @@
   </si>
   <si>
     <t>Noémi Villars-Amberg, Daniela Subotic</t>
+  </si>
+  <si>
+    <t>Wikidata Link</t>
+  </si>
+  <si>
+    <t>https://www.wikidata.org/wiki/Q20872991</t>
   </si>
 </sst>
 </file>
@@ -458,7 +463,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="8.5" customWidth="1"/>
@@ -469,7 +474,7 @@
     <col min="8" max="8" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -498,10 +503,13 @@
         <v>32</v>
       </c>
       <c r="J1" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="K1" s="8" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="87" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:11" ht="87" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
@@ -529,11 +537,14 @@
       <c r="I2" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="K2" s="8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
@@ -561,11 +572,12 @@
       <c r="I3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="9"/>
+      <c r="K3" s="8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
@@ -593,11 +605,12 @@
       <c r="I4" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="J4" s="9"/>
+      <c r="K4" s="8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="35.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:11" ht="35.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="3" t="s">
         <v>18</v>
       </c>
@@ -625,11 +638,12 @@
       <c r="I5" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="J5" s="9"/>
+      <c r="K5" s="8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="3" t="s">
         <v>21</v>
       </c>
@@ -657,7 +671,8 @@
       <c r="I6" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="9"/>
+      <c r="K6" s="8" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>